<commit_message>
Fix KPI basis, coverage and threshold findings (batch 8)
- Gross sales and discounts are on the same ex-VAT basis as returns and
  net sales, so the summary lines reconcile (C64).
- Variable cost is per unit sold everywhere, as in the founder's example
  (2,000 AMD per unit); renamed variableCostPerOrder to
  variableCostPerUnit (C65).
- Velocity uses only the days the imported sales cover (first to last
  sale, never past today); a gap is flagged DATA_NOT_COVERING_PERIOD (C49).
- LOW_VELOCITY_SAMPLE also applies to a SKU sold on fewer than 3 days,
  not only when the shop has fewer than 14 sales days (C48).
- Days of stock is compared with the thresholds unrounded; reports and
  texts round to one decimal (C85).
- The COGS_MISSING explanation says contribution is understated (C51).
- Sample report regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0139UNrTdUsr1c6bWNMxp85N
</commit_message>
<xml_diff>
--- a/retail-ai-platform/docs/samples/SAMPLE_weekly_report_synthetic_2026-09.xlsx
+++ b/retail-ai-platform/docs/samples/SAMPLE_weekly_report_synthetic_2026-09.xlsx
@@ -17,9 +17,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="158">
-  <si>
-    <t>Շաբաթական հաշվետվություն. Synthetic Sample 32073</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="157">
+  <si>
+    <t>Շաբաթական հաշվետվություն. Synthetic Sample 25036</t>
   </si>
   <si>
     <t>Շրջան</t>
@@ -31,7 +31,7 @@
     <t>Պատրաստված</t>
   </si>
   <si>
-    <t>12.10.2026 17:02</t>
+    <t>12.10.2026 17:11</t>
   </si>
   <si>
     <t>Ցուցանիշ</t>
@@ -46,7 +46,7 @@
     <t>Համախառն վաճառք (gross sales)</t>
   </si>
   <si>
-    <t>Վաճառքի տողերի գումար, զեղչից առաջ</t>
+    <t>Վաճառքի տողերի գումար, զեղչից առաջ, առանց ԱԱՀ, եթե ԱԱՀ-ի հիմքը հայտնի է</t>
   </si>
   <si>
     <t>Զեղչեր</t>
@@ -94,7 +94,7 @@
     <t>Փոփոխական ծախսեր (ենթադրություն)</t>
   </si>
   <si>
-    <t>Պատվերի ծախս × վաճառքի տողեր. հաստատել հաշվապահի հետ</t>
+    <t>Մեկ հատի ծախս × վաճառված հատեր. հաստատել հաշվապահի հետ</t>
   </si>
   <si>
     <t>Ծածկույթ (contribution)</t>
@@ -331,9 +331,6 @@
     <t>Սխալներ</t>
   </si>
   <si>
-    <t>12.10.2026 17:01</t>
-  </si>
-  <si>
     <t>committed</t>
   </si>
   <si>
@@ -451,7 +448,7 @@
     <t>Որոշում</t>
   </si>
   <si>
-    <t>9f8b50f0-933a-4e98-880e-2f6b5785a041</t>
+    <t>2aa617f2-81ef-439a-b9be-47c4298eb4df</t>
   </si>
   <si>
     <t>RESTOCK</t>
@@ -472,7 +469,7 @@
     <t>ACCEPTED / REJECTED / NEED_DATA</t>
   </si>
   <si>
-    <t>ac80abb8-0ded-45e4-8e7e-a20e2486a023</t>
+    <t>4f94798c-847a-46d0-ac5e-31b408038414</t>
   </si>
   <si>
     <t>AD_TEST</t>
@@ -481,10 +478,10 @@
     <t>MEDIUM</t>
   </si>
   <si>
-    <t>Ապրանք B-2001 (Ջինս կլասիկ 32)․ մաքուր գինը մոտ 39 122 դրամ/հատ է, ինքնարժեքը՝ 29 000, պատվերի փոփոխական ծախսը՝ 0։ Մինչև գովազդը մնում է մոտ 10 122 դրամ/հատ։ Առաջարկ՝ սահմանափակ փորձարկում, որտեղ մեկ վաճառքի ձեռքբերման արժեքը չգերազանցի 10 122 դրամը։ Նշագրված պատվերները դեռ չեն ապացուցում հավելյալ վաճառք։ Ենթադրություն՝ պատվերի փոփոխական ծախսը։ Բացակայում է՝ հավելյալ վաճառքի ապացույց (հնարավոր է միայն փորձարկմամբ)։ Շրջան՝ 01.09.2026 – 30.09.2026։ Վստահություն՝ միջին։ Պատասխանատու՝ մարքեթոլոգ։</t>
-  </si>
-  <si>
-    <t>a8dde007-e4af-4133-9a30-ecb6241feac3</t>
+    <t>Ապրանք B-2001 (Ջինս կլասիկ 32)․ մաքուր գինը մոտ 39 122 դրամ/հատ է, ինքնարժեքը՝ 29 000, մեկ հատի փոփոխական ծախսը՝ 0։ Մինչև գովազդը մնում է մոտ 10 122 դրամ/հատ։ Առաջարկ՝ սահմանափակ փորձարկում, որտեղ մեկ վաճառքի ձեռքբերման արժեքը չգերազանցի 10 122 դրամը։ Նշագրված պատվերները դեռ չեն ապացուցում հավելյալ վաճառք։ Ենթադրություն՝ մեկ հատի փոփոխական ծախսը (առաքում, միջնորդավճար, վերադարձ)։ Բացակայում է՝ հավելյալ վաճառքի ապացույց (հնարավոր է միայն փորձարկմամբ)։ Շրջան՝ 01.09.2026 – 30.09.2026։ Վստահություն՝ միջին։ Պատասխանատու՝ մարքեթոլոգ։</t>
+  </si>
+  <si>
+    <t>c5470a60-4f8a-4e9a-aeb1-f274daee1e6c</t>
   </si>
   <si>
     <t>SLOW_MOVER</t>
@@ -638,7 +635,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="n" s="6">
-        <v>5595000.0</v>
+        <v>4662500.0</v>
       </c>
       <c r="C6" t="s" s="5">
         <v>9</v>
@@ -649,7 +646,7 @@
         <v>10</v>
       </c>
       <c r="B7" t="n" s="6">
-        <v>77000.0</v>
+        <v>64166.67</v>
       </c>
       <c r="C7" t="s" s="5">
         <v>11</v>
@@ -1299,10 +1296,10 @@
         <v>82</v>
       </c>
       <c r="B3" t="s" s="4">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s" s="4">
         <v>104</v>
-      </c>
-      <c r="C3" t="s" s="4">
-        <v>105</v>
       </c>
       <c r="D3" t="n" s="7">
         <v>2.0</v>
@@ -1319,10 +1316,10 @@
         <v>88</v>
       </c>
       <c r="B4" t="s" s="4">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s" s="4">
         <v>104</v>
-      </c>
-      <c r="C4" t="s" s="4">
-        <v>105</v>
       </c>
       <c r="D4" t="n" s="7">
         <v>2.0</v>
@@ -1339,10 +1336,10 @@
         <v>94</v>
       </c>
       <c r="B5" t="s" s="4">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s" s="4">
         <v>104</v>
-      </c>
-      <c r="C5" t="s" s="4">
-        <v>105</v>
       </c>
       <c r="D5" t="n" s="7">
         <v>1.0</v>
@@ -1356,10 +1353,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="3">
+        <v>105</v>
+      </c>
+      <c r="B7" t="s" s="4">
         <v>106</v>
-      </c>
-      <c r="B7" t="s" s="4">
-        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1385,31 +1382,31 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="3">
+        <v>108</v>
+      </c>
+      <c r="B2" t="s" s="4">
         <v>109</v>
-      </c>
-      <c r="B2" t="s" s="4">
-        <v>110</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="3">
+        <v>110</v>
+      </c>
+      <c r="B3" t="s" s="4">
         <v>111</v>
       </c>
-      <c r="B3" t="s" s="4">
+      <c r="C3" t="s" s="5">
         <v>112</v>
-      </c>
-      <c r="C3" t="s" s="5">
-        <v>113</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="3">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B4" t="n" s="6">
         <v>300000.0</v>
@@ -1420,10 +1417,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="3">
+        <v>114</v>
+      </c>
+      <c r="B5" t="s" s="4">
         <v>115</v>
-      </c>
-      <c r="B5" t="s" s="4">
-        <v>116</v>
       </c>
       <c r="C5" t="s" s="5">
         <v>11</v>
@@ -1431,64 +1428,64 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="3">
+        <v>116</v>
+      </c>
+      <c r="B6" t="s" s="4">
         <v>117</v>
       </c>
-      <c r="B6" t="s" s="4">
+      <c r="C6" t="s" s="5">
         <v>118</v>
-      </c>
-      <c r="C6" t="s" s="5">
-        <v>119</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="3">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B7" t="s" s="8">
         <v>73</v>
       </c>
       <c r="C7" t="s" s="5">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B9" t="s" s="2">
         <v>100</v>
       </c>
       <c r="C9" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="D9" t="s" s="2">
         <v>123</v>
       </c>
-      <c r="D9" t="s" s="2">
+      <c r="E9" t="s" s="2">
         <v>124</v>
       </c>
-      <c r="E9" t="s" s="2">
+      <c r="F9" t="s" s="2">
         <v>125</v>
       </c>
-      <c r="F9" t="s" s="2">
+      <c r="G9" t="s" s="2">
         <v>126</v>
       </c>
-      <c r="G9" t="s" s="2">
+      <c r="H9" t="s" s="2">
         <v>127</v>
       </c>
-      <c r="H9" t="s" s="2">
-        <v>128</v>
-      </c>
       <c r="I9" t="s" s="2">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="4">
+        <v>128</v>
+      </c>
+      <c r="B10" t="s" s="4">
         <v>129</v>
       </c>
-      <c r="B10" t="s" s="4">
+      <c r="C10" t="s" s="4">
         <v>130</v>
-      </c>
-      <c r="C10" t="s" s="4">
-        <v>131</v>
       </c>
       <c r="D10" t="s" s="4">
         <v>11</v>
@@ -1506,21 +1503,21 @@
         <v>0.0</v>
       </c>
       <c r="I10" t="s" s="4">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="4">
+        <v>132</v>
+      </c>
+      <c r="B11" t="s" s="4">
         <v>133</v>
       </c>
-      <c r="B11" t="s" s="4">
+      <c r="C11" t="s" s="4">
         <v>134</v>
       </c>
-      <c r="C11" t="s" s="4">
+      <c r="D11" t="s" s="4">
         <v>135</v>
-      </c>
-      <c r="D11" t="s" s="4">
-        <v>136</v>
       </c>
       <c r="E11" t="n" s="6">
         <v>263700.0</v>
@@ -1535,21 +1532,21 @@
         <v>1.0</v>
       </c>
       <c r="I11" t="s" s="4">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="4">
+        <v>132</v>
+      </c>
+      <c r="B12" t="s" s="4">
         <v>133</v>
       </c>
-      <c r="B12" t="s" s="4">
+      <c r="C12" t="s" s="4">
         <v>134</v>
       </c>
-      <c r="C12" t="s" s="4">
-        <v>135</v>
-      </c>
       <c r="D12" t="s" s="4">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E12" t="n" s="6">
         <v>280000.0</v>
@@ -1564,7 +1561,7 @@
         <v>0.0</v>
       </c>
       <c r="I12" t="s" s="4">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -1589,7 +1586,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2">
@@ -1597,21 +1594,21 @@
         <v>46</v>
       </c>
       <c r="B2" t="s" s="4">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
+        <v>139</v>
+      </c>
+      <c r="B4" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="C4" t="s" s="2">
         <v>140</v>
       </c>
-      <c r="B4" t="s" s="2">
-        <v>122</v>
-      </c>
-      <c r="C4" t="s" s="2">
+      <c r="D4" t="s" s="2">
         <v>141</v>
-      </c>
-      <c r="D4" t="s" s="2">
-        <v>142</v>
       </c>
       <c r="E4" t="s" s="2">
         <v>100</v>
@@ -1623,85 +1620,85 @@
         <v>76</v>
       </c>
       <c r="H4" t="s" s="2">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="5">
+        <v>143</v>
+      </c>
+      <c r="B5" t="s" s="4">
         <v>144</v>
-      </c>
-      <c r="B5" t="s" s="4">
-        <v>145</v>
       </c>
       <c r="C5" t="s" s="4">
         <v>64</v>
       </c>
       <c r="D5" t="s" s="4">
+        <v>145</v>
+      </c>
+      <c r="E5" t="s" s="4">
         <v>146</v>
       </c>
-      <c r="E5" t="s" s="4">
+      <c r="F5" t="s" s="4">
         <v>147</v>
       </c>
-      <c r="F5" t="s" s="4">
+      <c r="G5" t="s" s="5">
         <v>148</v>
       </c>
-      <c r="G5" t="s" s="5">
+      <c r="H5" t="s" s="5">
         <v>149</v>
-      </c>
-      <c r="H5" t="s" s="5">
-        <v>150</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="5">
+        <v>150</v>
+      </c>
+      <c r="B6" t="s" s="4">
         <v>151</v>
-      </c>
-      <c r="B6" t="s" s="4">
-        <v>152</v>
       </c>
       <c r="C6" t="s" s="4">
         <v>62</v>
       </c>
       <c r="D6" t="s" s="4">
+        <v>152</v>
+      </c>
+      <c r="E6" t="s" s="4">
+        <v>146</v>
+      </c>
+      <c r="F6" t="s" s="4">
         <v>153</v>
       </c>
-      <c r="E6" t="s" s="4">
-        <v>147</v>
-      </c>
-      <c r="F6" t="s" s="4">
-        <v>154</v>
-      </c>
       <c r="G6" t="s" s="5">
+        <v>148</v>
+      </c>
+      <c r="H6" t="s" s="5">
         <v>149</v>
-      </c>
-      <c r="H6" t="s" s="5">
-        <v>150</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="5">
+        <v>154</v>
+      </c>
+      <c r="B7" t="s" s="4">
         <v>155</v>
-      </c>
-      <c r="B7" t="s" s="4">
-        <v>156</v>
       </c>
       <c r="C7" t="s" s="4">
         <v>71</v>
       </c>
       <c r="D7" t="s" s="4">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E7" t="s" s="4">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F7" t="s" s="4">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G7" t="s" s="5">
+        <v>148</v>
+      </c>
+      <c r="H7" t="s" s="5">
         <v>149</v>
-      </c>
-      <c r="H7" t="s" s="5">
-        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>